<commit_message>
Backup SellerOne control and runtime state 20260610
</commit_message>
<xml_diff>
--- a/plans/active/sellerone-endgame-command-center-2026-05-26/SellerOne_Endgame_Task_Board.xlsx
+++ b/plans/active/sellerone-endgame-command-center-2026-05-26/SellerOne_Endgame_Task_Board.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R39db7eadc43d4390"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Board" sheetId="2" r:id="R406534a40aa74845"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Result Checks" sheetId="3" r:id="R2d15cee6a2984ad8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goal Files" sheetId="4" r:id="Re81e92dcf7594c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="5" r:id="R874729010648422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R79cbe83f78634e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Board" sheetId="2" r:id="R8fa82e7b9aa749cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Result Checks" sheetId="3" r:id="R79bb4babd8ac4572"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goal Files" sheetId="4" r:id="R3bfde0874dae48d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="5" r:id="R75d316d68fde4c5a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,6 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+  </x:numFmts>
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
@@ -80,7 +83,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -106,6 +109,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2048,7 +2052,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97a62b0794c74ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1052a1d5d604234"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2299,28 +2303,32 @@
         <x:v>O-003</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Fresh market proof may require a safe H pause and then a later O rebuild.</x:v>
+        <x:v>Current evidence says H owns the market files; proof needs an approved elevated H isolation window before O can scan safely.</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>After approved H pause plus O candidate-only market scan, or next safe proof window</x:v>
+        <x:v>After Luke approves elevated H isolation pause plus O candidate-only market scan, or another safe H proof window</x:v>
       </x:c>
       <x:c r="E8" t="str">
         <x:v>out/systems/O/history/ and out/systems/O/live/restock_profit_checks_live.csv</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>59 candidates either receive native market proof or remain held with clear missing-data reasons</x:v>
+        <x:v>59 candidates either receive native market proof or remain held with clear missing-data reasons; H ownership is restored after the scan</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>Keep O buy rows blocked and inspect H/O market ownership first</x:v>
+        <x:v>Keep O buy rows blocked and inspect H/O market ownership first; do not run the market scan while an H lock has a live heartbeat</x:v>
       </x:c>
       <x:c r="H8" t="str">
         <x:v>Joint</x:v>
       </x:c>
       <x:c r="I8" t="str">
-        <x:v>Waiting for proof window</x:v>
-      </x:c>
-      <x:c r="J8"/>
-      <x:c r="K8"/>
+        <x:v>Waiting for user decision</x:v>
+      </x:c>
+      <x:c r="J8" s="15" t="str">
+        <x:v>checked 2026-05-26T10:32:33Z</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>O-003 checked: 59 ready candidates still exist; all 59 matched profit rows use LEGACY_PURCHASE_LIST_ROI_BACKSOLVE; H active lock run_id=20260526T100940Z pid=24476 heartbeat=2026-05-26T10:32:20Z.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="I2:I7">
@@ -2335,7 +2343,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ffd3303539e4548"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0033a95df0874ff5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2495,7 +2503,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2152b4499f44193"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fabd9d6f04e4398"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>